<commit_message>
New Schema Fields: Osage Nation Final Report Completion Deepening
</commit_message>
<xml_diff>
--- a/src/ogrre_data_cleaning/processor_schemas/Osage Nation Schema.xlsx
+++ b/src/ogrre_data_cleaning/processor_schemas/Osage Nation Schema.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="962" uniqueCount="270">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="962" uniqueCount="269">
   <si>
     <t>Processor Type</t>
   </si>
@@ -119,15 +119,15 @@
     <t>V1_5-07</t>
   </si>
   <si>
+    <t>2c4d1ab39b312baf</t>
+  </si>
+  <si>
+    <t>V1_5-08</t>
+  </si>
+  <si>
     <t>primary</t>
   </si>
   <si>
-    <t>2c4d1ab39b312baf</t>
-  </si>
-  <si>
-    <t>V1_5-08</t>
-  </si>
-  <si>
     <t>e90c3d16d03e7c61</t>
   </si>
   <si>
@@ -816,9 +816,6 @@
   </si>
   <si>
     <t>Shot_Size</t>
-  </si>
-  <si>
-    <t>Shot_Qts</t>
   </si>
   <si>
     <t>Gas_Initial_Flow_Sand_From</t>
@@ -1621,9 +1618,7 @@
       <c r="D10" s="4">
         <v>0.867</v>
       </c>
-      <c r="E10" s="4" t="s">
-        <v>33</v>
-      </c>
+      <c r="E10" s="4"/>
       <c r="F10" s="5">
         <v>172.0</v>
       </c>
@@ -1640,7 +1635,7 @@
         <v>15</v>
       </c>
       <c r="K10" s="4" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="11">
@@ -1651,12 +1646,14 @@
         <v>12</v>
       </c>
       <c r="C11" s="9" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D11" s="9">
         <v>0.88</v>
       </c>
-      <c r="E11" s="9"/>
+      <c r="E11" s="9" t="s">
+        <v>35</v>
+      </c>
       <c r="F11" s="10">
         <v>175.0</v>
       </c>
@@ -1820,7 +1817,7 @@
         <v>0.926</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="F16" s="5">
         <v>96.0</v>
@@ -1855,7 +1852,7 @@
         <v>0.877</v>
       </c>
       <c r="E17" s="9" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="F17" s="10">
         <v>808.0</v>
@@ -7609,7 +7606,9 @@
       <c r="V2" s="3">
         <v>0.775</v>
       </c>
-      <c r="W2" s="3"/>
+      <c r="W2" s="7">
+        <v>0.77</v>
+      </c>
       <c r="X2" s="3">
         <v>0.765</v>
       </c>
@@ -7653,7 +7652,9 @@
       <c r="T3" s="8"/>
       <c r="U3" s="8"/>
       <c r="V3" s="8"/>
-      <c r="W3" s="8"/>
+      <c r="W3" s="12">
+        <v>0.948</v>
+      </c>
       <c r="X3" s="8"/>
     </row>
     <row r="4">
@@ -7695,7 +7696,9 @@
       <c r="T4" s="3"/>
       <c r="U4" s="3"/>
       <c r="V4" s="3"/>
-      <c r="W4" s="3"/>
+      <c r="W4" s="7">
+        <v>0.964</v>
+      </c>
       <c r="X4" s="3"/>
     </row>
     <row r="5">
@@ -7737,7 +7740,9 @@
       <c r="T5" s="8"/>
       <c r="U5" s="8"/>
       <c r="V5" s="8"/>
-      <c r="W5" s="8"/>
+      <c r="W5" s="12">
+        <v>0.951</v>
+      </c>
       <c r="X5" s="8"/>
     </row>
     <row r="6">
@@ -7779,7 +7784,9 @@
       <c r="T6" s="3"/>
       <c r="U6" s="3"/>
       <c r="V6" s="3"/>
-      <c r="W6" s="3"/>
+      <c r="W6" s="7">
+        <v>0.956</v>
+      </c>
       <c r="X6" s="3"/>
     </row>
     <row r="7">
@@ -7789,60 +7796,40 @@
       <c r="B7" s="8" t="s">
         <v>171</v>
       </c>
-      <c r="C7" s="8">
+      <c r="C7" s="12">
         <v>6.0</v>
       </c>
-      <c r="D7" s="8" t="s">
-        <v>111</v>
-      </c>
-      <c r="E7" s="8" t="s">
-        <v>111</v>
-      </c>
-      <c r="F7" s="8"/>
-      <c r="G7" s="8" t="s">
+      <c r="D7" s="12" t="s">
+        <v>109</v>
+      </c>
+      <c r="E7" s="21"/>
+      <c r="F7" s="21"/>
+      <c r="G7" s="12" t="s">
         <v>105</v>
       </c>
-      <c r="H7" s="8" t="s">
+      <c r="H7" s="12" t="s">
         <v>106</v>
       </c>
-      <c r="I7" s="8"/>
-      <c r="J7" s="8" t="s">
+      <c r="I7" s="21"/>
+      <c r="J7" s="12" t="s">
         <v>107</v>
       </c>
-      <c r="K7" s="8" t="s">
+      <c r="K7" s="12" t="s">
         <v>108</v>
       </c>
-      <c r="L7" s="8"/>
-      <c r="M7" s="8"/>
+      <c r="L7" s="21"/>
+      <c r="M7" s="21"/>
       <c r="N7" s="21"/>
-      <c r="O7" s="8">
-        <v>0.667</v>
-      </c>
-      <c r="P7" s="8">
-        <v>0.81</v>
-      </c>
-      <c r="Q7" s="8">
-        <v>0.743</v>
-      </c>
-      <c r="R7" s="8">
-        <v>0.889</v>
-      </c>
-      <c r="S7" s="8">
-        <v>0.804</v>
-      </c>
-      <c r="T7" s="8">
-        <v>0.721</v>
-      </c>
-      <c r="U7" s="8">
-        <v>0.699</v>
-      </c>
-      <c r="V7" s="8">
-        <v>0.791</v>
-      </c>
-      <c r="W7" s="8"/>
-      <c r="X7" s="8">
-        <v>0.794</v>
-      </c>
+      <c r="O7" s="21"/>
+      <c r="P7" s="21"/>
+      <c r="Q7" s="21"/>
+      <c r="R7" s="21"/>
+      <c r="S7" s="21"/>
+      <c r="T7" s="21"/>
+      <c r="U7" s="21"/>
+      <c r="V7" s="21"/>
+      <c r="W7" s="12"/>
+      <c r="X7" s="21"/>
     </row>
     <row r="8">
       <c r="A8" s="3" t="s">
@@ -7851,59 +7838,61 @@
       <c r="B8" s="3" t="s">
         <v>171</v>
       </c>
-      <c r="C8" s="3">
+      <c r="C8" s="7">
         <v>7.0</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="F8" s="3"/>
       <c r="G8" s="3" t="s">
-        <v>115</v>
+        <v>105</v>
       </c>
       <c r="H8" s="3" t="s">
         <v>106</v>
       </c>
       <c r="I8" s="3"/>
       <c r="J8" s="3" t="s">
-        <v>121</v>
+        <v>107</v>
       </c>
       <c r="K8" s="3" t="s">
-        <v>116</v>
+        <v>108</v>
       </c>
       <c r="L8" s="3"/>
       <c r="M8" s="3"/>
       <c r="N8" s="19"/>
       <c r="O8" s="3">
-        <v>0.933</v>
+        <v>0.667</v>
       </c>
       <c r="P8" s="3">
-        <v>0.96</v>
+        <v>0.81</v>
       </c>
       <c r="Q8" s="3">
-        <v>1.0</v>
+        <v>0.743</v>
       </c>
       <c r="R8" s="3">
-        <v>0.986</v>
+        <v>0.889</v>
       </c>
       <c r="S8" s="3">
-        <v>0.993</v>
+        <v>0.804</v>
       </c>
       <c r="T8" s="3">
-        <v>0.956</v>
+        <v>0.721</v>
       </c>
       <c r="U8" s="3">
-        <v>0.971</v>
+        <v>0.699</v>
       </c>
       <c r="V8" s="3">
-        <v>1.0</v>
-      </c>
-      <c r="W8" s="3"/>
+        <v>0.791</v>
+      </c>
+      <c r="W8" s="7">
+        <v>0.873</v>
+      </c>
       <c r="X8" s="3">
-        <v>0.981</v>
+        <v>0.794</v>
       </c>
     </row>
     <row r="9">
@@ -7913,34 +7902,34 @@
       <c r="B9" s="8" t="s">
         <v>171</v>
       </c>
-      <c r="C9" s="8">
+      <c r="C9" s="12">
         <v>8.0</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="F9" s="8"/>
       <c r="G9" s="8" t="s">
-        <v>105</v>
+        <v>115</v>
       </c>
       <c r="H9" s="8" t="s">
         <v>106</v>
       </c>
       <c r="I9" s="8"/>
       <c r="J9" s="8" t="s">
-        <v>107</v>
+        <v>121</v>
       </c>
       <c r="K9" s="8" t="s">
-        <v>108</v>
+        <v>116</v>
       </c>
       <c r="L9" s="8"/>
       <c r="M9" s="8"/>
       <c r="N9" s="21"/>
       <c r="O9" s="8">
-        <v>0.867</v>
+        <v>0.933</v>
       </c>
       <c r="P9" s="8">
         <v>0.96</v>
@@ -7949,23 +7938,25 @@
         <v>1.0</v>
       </c>
       <c r="R9" s="8">
-        <v>0.971</v>
+        <v>0.986</v>
       </c>
       <c r="S9" s="8">
         <v>0.993</v>
       </c>
       <c r="T9" s="8">
+        <v>0.956</v>
+      </c>
+      <c r="U9" s="8">
         <v>0.971</v>
       </c>
-      <c r="U9" s="8">
-        <v>0.941</v>
-      </c>
       <c r="V9" s="8">
+        <v>1.0</v>
+      </c>
+      <c r="W9" s="12">
+        <v>0.994</v>
+      </c>
+      <c r="X9" s="8">
         <v>0.981</v>
-      </c>
-      <c r="W9" s="8"/>
-      <c r="X9" s="8">
-        <v>0.968</v>
       </c>
     </row>
     <row r="10">
@@ -7975,14 +7966,14 @@
       <c r="B10" s="3" t="s">
         <v>171</v>
       </c>
-      <c r="C10" s="3">
+      <c r="C10" s="7">
         <v>9.0</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="F10" s="3"/>
       <c r="G10" s="3" t="s">
@@ -8002,32 +7993,34 @@
       <c r="M10" s="3"/>
       <c r="N10" s="19"/>
       <c r="O10" s="3">
-        <v>0.966</v>
+        <v>0.867</v>
       </c>
       <c r="P10" s="3">
-        <v>1.0</v>
+        <v>0.96</v>
       </c>
       <c r="Q10" s="3">
         <v>1.0</v>
       </c>
       <c r="R10" s="3">
-        <v>0.957</v>
+        <v>0.971</v>
       </c>
       <c r="S10" s="3">
+        <v>0.993</v>
+      </c>
+      <c r="T10" s="3">
+        <v>0.971</v>
+      </c>
+      <c r="U10" s="3">
         <v>0.941</v>
       </c>
-      <c r="T10" s="3">
-        <v>0.964</v>
-      </c>
-      <c r="U10" s="3">
-        <v>0.913</v>
-      </c>
       <c r="V10" s="3">
-        <v>0.931</v>
-      </c>
-      <c r="W10" s="3"/>
+        <v>0.981</v>
+      </c>
+      <c r="W10" s="7">
+        <v>0.982</v>
+      </c>
       <c r="X10" s="3">
-        <v>0.937</v>
+        <v>0.968</v>
       </c>
     </row>
     <row r="11">
@@ -8037,36 +8030,34 @@
       <c r="B11" s="8" t="s">
         <v>171</v>
       </c>
-      <c r="C11" s="8">
+      <c r="C11" s="12">
         <v>10.0</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>177</v>
+        <v>119</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>178</v>
-      </c>
-      <c r="F11" s="8" t="s">
-        <v>179</v>
-      </c>
+        <v>120</v>
+      </c>
+      <c r="F11" s="8"/>
       <c r="G11" s="8" t="s">
-        <v>115</v>
+        <v>105</v>
       </c>
       <c r="H11" s="8" t="s">
         <v>106</v>
       </c>
-      <c r="I11" s="21"/>
+      <c r="I11" s="8"/>
       <c r="J11" s="8" t="s">
-        <v>134</v>
+        <v>107</v>
       </c>
       <c r="K11" s="8" t="s">
-        <v>135</v>
-      </c>
-      <c r="L11" s="21"/>
-      <c r="M11" s="21"/>
+        <v>108</v>
+      </c>
+      <c r="L11" s="8"/>
+      <c r="M11" s="8"/>
       <c r="N11" s="21"/>
       <c r="O11" s="8">
-        <v>1.0</v>
+        <v>0.966</v>
       </c>
       <c r="P11" s="8">
         <v>1.0</v>
@@ -8075,23 +8066,25 @@
         <v>1.0</v>
       </c>
       <c r="R11" s="8">
-        <v>0.977</v>
+        <v>0.957</v>
       </c>
       <c r="S11" s="8">
-        <v>0.977</v>
+        <v>0.941</v>
       </c>
       <c r="T11" s="8">
-        <v>0.97</v>
+        <v>0.964</v>
       </c>
       <c r="U11" s="8">
-        <v>0.985</v>
+        <v>0.913</v>
       </c>
       <c r="V11" s="8">
-        <v>0.987</v>
-      </c>
-      <c r="W11" s="8"/>
+        <v>0.931</v>
+      </c>
+      <c r="W11" s="12">
+        <v>0.929</v>
+      </c>
       <c r="X11" s="8">
-        <v>0.974</v>
+        <v>0.937</v>
       </c>
     </row>
     <row r="12">
@@ -8101,61 +8094,63 @@
       <c r="B12" s="3" t="s">
         <v>171</v>
       </c>
-      <c r="C12" s="3">
+      <c r="C12" s="7">
         <v>11.0</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>105</v>
+        <v>115</v>
       </c>
       <c r="H12" s="3" t="s">
         <v>106</v>
       </c>
       <c r="I12" s="19"/>
       <c r="J12" s="3" t="s">
-        <v>107</v>
+        <v>134</v>
       </c>
       <c r="K12" s="3" t="s">
-        <v>108</v>
+        <v>135</v>
       </c>
       <c r="L12" s="19"/>
       <c r="M12" s="19"/>
       <c r="N12" s="19"/>
       <c r="O12" s="3">
-        <v>0.69</v>
+        <v>1.0</v>
       </c>
       <c r="P12" s="3">
-        <v>0.5</v>
+        <v>1.0</v>
       </c>
       <c r="Q12" s="3">
-        <v>0.602</v>
+        <v>1.0</v>
       </c>
       <c r="R12" s="3">
-        <v>0.672</v>
+        <v>0.977</v>
       </c>
       <c r="S12" s="3">
-        <v>0.632</v>
+        <v>0.977</v>
       </c>
       <c r="T12" s="3">
-        <v>0.567</v>
+        <v>0.97</v>
       </c>
       <c r="U12" s="3">
-        <v>0.696</v>
+        <v>0.985</v>
       </c>
       <c r="V12" s="3">
-        <v>0.632</v>
-      </c>
-      <c r="W12" s="3"/>
+        <v>0.987</v>
+      </c>
+      <c r="W12" s="7">
+        <v>0.994</v>
+      </c>
       <c r="X12" s="3">
-        <v>0.611</v>
+        <v>0.974</v>
       </c>
     </row>
     <row r="13">
@@ -8165,61 +8160,63 @@
       <c r="B13" s="8" t="s">
         <v>171</v>
       </c>
-      <c r="C13" s="8">
+      <c r="C13" s="12">
         <v>12.0</v>
       </c>
       <c r="D13" s="8" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="F13" s="8" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="G13" s="8" t="s">
-        <v>115</v>
+        <v>105</v>
       </c>
       <c r="H13" s="8" t="s">
         <v>106</v>
       </c>
       <c r="I13" s="21"/>
       <c r="J13" s="8" t="s">
-        <v>134</v>
+        <v>107</v>
       </c>
       <c r="K13" s="8" t="s">
-        <v>135</v>
+        <v>108</v>
       </c>
       <c r="L13" s="21"/>
       <c r="M13" s="21"/>
       <c r="N13" s="21"/>
       <c r="O13" s="8">
-        <v>1.0</v>
+        <v>0.69</v>
       </c>
       <c r="P13" s="8">
-        <v>0.979</v>
+        <v>0.5</v>
       </c>
       <c r="Q13" s="8">
-        <v>0.989</v>
+        <v>0.602</v>
       </c>
       <c r="R13" s="8">
-        <v>1.0</v>
+        <v>0.672</v>
       </c>
       <c r="S13" s="8">
-        <v>0.992</v>
+        <v>0.632</v>
       </c>
       <c r="T13" s="8">
-        <v>0.992</v>
+        <v>0.567</v>
       </c>
       <c r="U13" s="8">
-        <v>1.0</v>
+        <v>0.696</v>
       </c>
       <c r="V13" s="8">
-        <v>1.0</v>
-      </c>
-      <c r="W13" s="8"/>
+        <v>0.632</v>
+      </c>
+      <c r="W13" s="12">
+        <v>0.65</v>
+      </c>
       <c r="X13" s="8">
-        <v>1.0</v>
+        <v>0.611</v>
       </c>
     </row>
     <row r="14">
@@ -8229,61 +8226,63 @@
       <c r="B14" s="3" t="s">
         <v>171</v>
       </c>
-      <c r="C14" s="3">
+      <c r="C14" s="7">
         <v>13.0</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>187</v>
+        <v>179</v>
       </c>
       <c r="G14" s="3" t="s">
-        <v>105</v>
+        <v>115</v>
       </c>
       <c r="H14" s="3" t="s">
         <v>106</v>
       </c>
       <c r="I14" s="19"/>
       <c r="J14" s="3" t="s">
-        <v>107</v>
+        <v>134</v>
       </c>
       <c r="K14" s="3" t="s">
-        <v>108</v>
+        <v>135</v>
       </c>
       <c r="L14" s="19"/>
       <c r="M14" s="19"/>
       <c r="N14" s="19"/>
       <c r="O14" s="3">
-        <v>0.571</v>
+        <v>1.0</v>
       </c>
       <c r="P14" s="3">
-        <v>0.609</v>
+        <v>0.979</v>
       </c>
       <c r="Q14" s="3">
-        <v>0.554</v>
+        <v>0.989</v>
       </c>
       <c r="R14" s="3">
-        <v>0.713</v>
+        <v>1.0</v>
       </c>
       <c r="S14" s="3">
-        <v>0.61</v>
+        <v>0.992</v>
       </c>
       <c r="T14" s="3">
-        <v>0.677</v>
+        <v>0.992</v>
       </c>
       <c r="U14" s="3">
-        <v>0.662</v>
+        <v>1.0</v>
       </c>
       <c r="V14" s="3">
-        <v>0.634</v>
-      </c>
-      <c r="W14" s="3"/>
+        <v>1.0</v>
+      </c>
+      <c r="W14" s="7">
+        <v>1.0</v>
+      </c>
       <c r="X14" s="3">
-        <v>0.634</v>
+        <v>1.0</v>
       </c>
     </row>
     <row r="15">
@@ -8293,42 +8292,64 @@
       <c r="B15" s="8" t="s">
         <v>171</v>
       </c>
-      <c r="C15" s="8">
+      <c r="C15" s="12">
         <v>14.0</v>
       </c>
       <c r="D15" s="8" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>189</v>
-      </c>
-      <c r="F15" s="8"/>
-      <c r="G15" s="12" t="s">
+        <v>186</v>
+      </c>
+      <c r="F15" s="8" t="s">
+        <v>187</v>
+      </c>
+      <c r="G15" s="8" t="s">
         <v>105</v>
       </c>
       <c r="H15" s="8" t="s">
         <v>106</v>
       </c>
       <c r="I15" s="21"/>
-      <c r="J15" s="12" t="s">
-        <v>134</v>
+      <c r="J15" s="8" t="s">
+        <v>107</v>
       </c>
       <c r="K15" s="8" t="s">
-        <v>135</v>
+        <v>108</v>
       </c>
       <c r="L15" s="21"/>
       <c r="M15" s="21"/>
       <c r="N15" s="21"/>
-      <c r="O15" s="8"/>
-      <c r="P15" s="8"/>
-      <c r="Q15" s="8"/>
-      <c r="R15" s="8"/>
-      <c r="S15" s="8"/>
-      <c r="T15" s="8"/>
-      <c r="U15" s="8"/>
-      <c r="V15" s="8"/>
-      <c r="W15" s="8"/>
-      <c r="X15" s="8"/>
+      <c r="O15" s="8">
+        <v>0.571</v>
+      </c>
+      <c r="P15" s="8">
+        <v>0.609</v>
+      </c>
+      <c r="Q15" s="8">
+        <v>0.554</v>
+      </c>
+      <c r="R15" s="8">
+        <v>0.713</v>
+      </c>
+      <c r="S15" s="8">
+        <v>0.61</v>
+      </c>
+      <c r="T15" s="8">
+        <v>0.677</v>
+      </c>
+      <c r="U15" s="8">
+        <v>0.662</v>
+      </c>
+      <c r="V15" s="8">
+        <v>0.634</v>
+      </c>
+      <c r="W15" s="12">
+        <v>0.594</v>
+      </c>
+      <c r="X15" s="8">
+        <v>0.634</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="s">
@@ -8337,18 +8358,16 @@
       <c r="B16" s="3" t="s">
         <v>171</v>
       </c>
-      <c r="C16" s="3">
+      <c r="C16" s="7">
         <v>15.0</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>191</v>
-      </c>
-      <c r="F16" s="3" t="s">
-        <v>179</v>
-      </c>
+        <v>189</v>
+      </c>
+      <c r="F16" s="3"/>
       <c r="G16" s="7" t="s">
         <v>105</v>
       </c>
@@ -8356,7 +8375,7 @@
         <v>106</v>
       </c>
       <c r="I16" s="19"/>
-      <c r="J16" s="3" t="s">
+      <c r="J16" s="7" t="s">
         <v>134</v>
       </c>
       <c r="K16" s="3" t="s">
@@ -8365,34 +8384,18 @@
       <c r="L16" s="19"/>
       <c r="M16" s="19"/>
       <c r="N16" s="19"/>
-      <c r="O16" s="3">
-        <v>0.741</v>
-      </c>
-      <c r="P16" s="3">
-        <v>0.837</v>
-      </c>
-      <c r="Q16" s="3">
-        <v>0.82</v>
-      </c>
-      <c r="R16" s="3">
-        <v>0.774</v>
-      </c>
-      <c r="S16" s="3">
-        <v>0.778</v>
-      </c>
-      <c r="T16" s="3">
-        <v>0.76</v>
-      </c>
-      <c r="U16" s="3">
-        <v>0.811</v>
-      </c>
-      <c r="V16" s="3">
-        <v>0.94</v>
-      </c>
-      <c r="W16" s="3"/>
-      <c r="X16" s="3">
-        <v>0.877</v>
-      </c>
+      <c r="O16" s="3"/>
+      <c r="P16" s="3"/>
+      <c r="Q16" s="3"/>
+      <c r="R16" s="3"/>
+      <c r="S16" s="3"/>
+      <c r="T16" s="3"/>
+      <c r="U16" s="3"/>
+      <c r="V16" s="3"/>
+      <c r="W16" s="7">
+        <v>0.968</v>
+      </c>
+      <c r="X16" s="3"/>
     </row>
     <row r="17">
       <c r="A17" s="8" t="s">
@@ -8401,42 +8404,64 @@
       <c r="B17" s="8" t="s">
         <v>171</v>
       </c>
-      <c r="C17" s="8">
+      <c r="C17" s="12">
         <v>16.0</v>
       </c>
       <c r="D17" s="8" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="E17" s="8" t="s">
-        <v>193</v>
-      </c>
-      <c r="F17" s="8"/>
-      <c r="G17" s="8" t="s">
-        <v>115</v>
+        <v>191</v>
+      </c>
+      <c r="F17" s="8" t="s">
+        <v>179</v>
+      </c>
+      <c r="G17" s="12" t="s">
+        <v>105</v>
       </c>
       <c r="H17" s="8" t="s">
         <v>106</v>
       </c>
-      <c r="I17" s="8"/>
-      <c r="J17" s="12" t="s">
+      <c r="I17" s="21"/>
+      <c r="J17" s="8" t="s">
         <v>134</v>
       </c>
       <c r="K17" s="8" t="s">
         <v>135</v>
       </c>
-      <c r="L17" s="8"/>
-      <c r="M17" s="8"/>
+      <c r="L17" s="21"/>
+      <c r="M17" s="21"/>
       <c r="N17" s="21"/>
-      <c r="O17" s="8"/>
-      <c r="P17" s="8"/>
-      <c r="Q17" s="8"/>
-      <c r="R17" s="8"/>
-      <c r="S17" s="8"/>
-      <c r="T17" s="8"/>
-      <c r="U17" s="8"/>
-      <c r="V17" s="8"/>
-      <c r="W17" s="8"/>
-      <c r="X17" s="8"/>
+      <c r="O17" s="8">
+        <v>0.741</v>
+      </c>
+      <c r="P17" s="8">
+        <v>0.837</v>
+      </c>
+      <c r="Q17" s="8">
+        <v>0.82</v>
+      </c>
+      <c r="R17" s="8">
+        <v>0.774</v>
+      </c>
+      <c r="S17" s="8">
+        <v>0.778</v>
+      </c>
+      <c r="T17" s="8">
+        <v>0.76</v>
+      </c>
+      <c r="U17" s="8">
+        <v>0.811</v>
+      </c>
+      <c r="V17" s="8">
+        <v>0.94</v>
+      </c>
+      <c r="W17" s="12">
+        <v>0.909</v>
+      </c>
+      <c r="X17" s="8">
+        <v>0.877</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="s">
@@ -8445,60 +8470,44 @@
       <c r="B18" s="3" t="s">
         <v>171</v>
       </c>
-      <c r="C18" s="3">
+      <c r="C18" s="7">
         <v>17.0</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="F18" s="3"/>
       <c r="G18" s="3" t="s">
-        <v>125</v>
+        <v>115</v>
       </c>
       <c r="H18" s="3" t="s">
         <v>106</v>
       </c>
       <c r="I18" s="3"/>
-      <c r="J18" s="3" t="s">
-        <v>126</v>
+      <c r="J18" s="7" t="s">
+        <v>134</v>
       </c>
       <c r="K18" s="3" t="s">
-        <v>127</v>
+        <v>135</v>
       </c>
       <c r="L18" s="3"/>
       <c r="M18" s="3"/>
       <c r="N18" s="19"/>
-      <c r="O18" s="3">
-        <v>0.846</v>
-      </c>
-      <c r="P18" s="3">
-        <v>0.818</v>
-      </c>
-      <c r="Q18" s="3">
-        <v>0.905</v>
-      </c>
-      <c r="R18" s="3">
-        <v>0.917</v>
-      </c>
-      <c r="S18" s="3">
-        <v>0.913</v>
-      </c>
-      <c r="T18" s="3">
-        <v>0.846</v>
-      </c>
-      <c r="U18" s="3">
-        <v>0.924</v>
-      </c>
-      <c r="V18" s="3">
-        <v>0.887</v>
-      </c>
-      <c r="W18" s="3"/>
-      <c r="X18" s="3">
-        <v>0.887</v>
-      </c>
+      <c r="O18" s="3"/>
+      <c r="P18" s="3"/>
+      <c r="Q18" s="3"/>
+      <c r="R18" s="3"/>
+      <c r="S18" s="3"/>
+      <c r="T18" s="3"/>
+      <c r="U18" s="3"/>
+      <c r="V18" s="3"/>
+      <c r="W18" s="7">
+        <v>0.871</v>
+      </c>
+      <c r="X18" s="3"/>
     </row>
     <row r="19">
       <c r="A19" s="8" t="s">
@@ -8507,14 +8516,14 @@
       <c r="B19" s="8" t="s">
         <v>171</v>
       </c>
-      <c r="C19" s="8">
+      <c r="C19" s="12">
         <v>18.0</v>
       </c>
       <c r="D19" s="8" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="E19" s="8" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="F19" s="8"/>
       <c r="G19" s="8" t="s">
@@ -8534,32 +8543,34 @@
       <c r="M19" s="8"/>
       <c r="N19" s="21"/>
       <c r="O19" s="8">
-        <v>0.889</v>
+        <v>0.846</v>
       </c>
       <c r="P19" s="8">
-        <v>0.773</v>
+        <v>0.818</v>
       </c>
       <c r="Q19" s="8">
-        <v>0.831</v>
+        <v>0.905</v>
       </c>
       <c r="R19" s="8">
-        <v>0.857</v>
+        <v>0.917</v>
       </c>
       <c r="S19" s="8">
-        <v>0.843</v>
+        <v>0.913</v>
       </c>
       <c r="T19" s="8">
-        <v>0.819</v>
+        <v>0.846</v>
       </c>
       <c r="U19" s="8">
-        <v>0.869</v>
+        <v>0.924</v>
       </c>
       <c r="V19" s="8">
-        <v>0.851</v>
-      </c>
-      <c r="W19" s="8"/>
+        <v>0.887</v>
+      </c>
+      <c r="W19" s="12">
+        <v>0.904</v>
+      </c>
       <c r="X19" s="8">
-        <v>0.838</v>
+        <v>0.887</v>
       </c>
     </row>
     <row r="20">
@@ -8569,42 +8580,62 @@
       <c r="B20" s="3" t="s">
         <v>171</v>
       </c>
-      <c r="C20" s="3">
+      <c r="C20" s="7">
         <v>19.0</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>199</v>
-      </c>
-      <c r="F20" s="19"/>
+        <v>197</v>
+      </c>
+      <c r="F20" s="3"/>
       <c r="G20" s="3" t="s">
-        <v>200</v>
+        <v>125</v>
       </c>
       <c r="H20" s="3" t="s">
         <v>106</v>
       </c>
-      <c r="I20" s="19"/>
-      <c r="J20" s="7" t="s">
-        <v>107</v>
-      </c>
-      <c r="K20" s="7" t="s">
-        <v>108</v>
-      </c>
-      <c r="L20" s="19"/>
-      <c r="M20" s="19"/>
+      <c r="I20" s="3"/>
+      <c r="J20" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="K20" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="L20" s="3"/>
+      <c r="M20" s="3"/>
       <c r="N20" s="19"/>
-      <c r="O20" s="19"/>
-      <c r="P20" s="19"/>
-      <c r="Q20" s="19"/>
-      <c r="R20" s="19"/>
-      <c r="S20" s="19"/>
-      <c r="T20" s="19"/>
-      <c r="U20" s="19"/>
-      <c r="V20" s="19"/>
-      <c r="W20" s="19"/>
-      <c r="X20" s="19"/>
+      <c r="O20" s="3">
+        <v>0.889</v>
+      </c>
+      <c r="P20" s="3">
+        <v>0.773</v>
+      </c>
+      <c r="Q20" s="3">
+        <v>0.831</v>
+      </c>
+      <c r="R20" s="3">
+        <v>0.857</v>
+      </c>
+      <c r="S20" s="3">
+        <v>0.843</v>
+      </c>
+      <c r="T20" s="3">
+        <v>0.819</v>
+      </c>
+      <c r="U20" s="3">
+        <v>0.869</v>
+      </c>
+      <c r="V20" s="3">
+        <v>0.851</v>
+      </c>
+      <c r="W20" s="7">
+        <v>0.855</v>
+      </c>
+      <c r="X20" s="3">
+        <v>0.838</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="8" t="s">
@@ -8613,60 +8644,44 @@
       <c r="B21" s="8" t="s">
         <v>171</v>
       </c>
-      <c r="C21" s="8">
+      <c r="C21" s="12">
         <v>20.0</v>
       </c>
       <c r="D21" s="8" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="E21" s="8" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="F21" s="21"/>
-      <c r="G21" s="21" t="s">
-        <v>144</v>
+      <c r="G21" s="8" t="s">
+        <v>200</v>
       </c>
       <c r="H21" s="8" t="s">
-        <v>145</v>
+        <v>106</v>
       </c>
       <c r="I21" s="21"/>
-      <c r="J21" s="21" t="s">
-        <v>146</v>
-      </c>
-      <c r="K21" s="21" t="s">
+      <c r="J21" s="12" t="s">
+        <v>107</v>
+      </c>
+      <c r="K21" s="12" t="s">
         <v>108</v>
       </c>
       <c r="L21" s="21"/>
       <c r="M21" s="21"/>
       <c r="N21" s="21"/>
-      <c r="O21" s="8">
-        <v>0.699</v>
-      </c>
-      <c r="P21" s="8">
-        <v>0.74</v>
-      </c>
-      <c r="Q21" s="8">
-        <v>0.812</v>
-      </c>
-      <c r="R21" s="8">
-        <v>0.859</v>
-      </c>
-      <c r="S21" s="8">
-        <v>0.863</v>
-      </c>
-      <c r="T21" s="8">
-        <v>0.819</v>
-      </c>
-      <c r="U21" s="8">
-        <v>0.838</v>
-      </c>
-      <c r="V21" s="8">
-        <v>0.861</v>
-      </c>
-      <c r="W21" s="8"/>
-      <c r="X21" s="8">
-        <v>0.838</v>
-      </c>
+      <c r="O21" s="21"/>
+      <c r="P21" s="21"/>
+      <c r="Q21" s="21"/>
+      <c r="R21" s="21"/>
+      <c r="S21" s="21"/>
+      <c r="T21" s="21"/>
+      <c r="U21" s="21"/>
+      <c r="V21" s="21"/>
+      <c r="W21" s="12">
+        <v>1.0</v>
+      </c>
+      <c r="X21" s="21"/>
     </row>
     <row r="22">
       <c r="A22" s="3" t="s">
@@ -8675,61 +8690,61 @@
       <c r="B22" s="3" t="s">
         <v>171</v>
       </c>
-      <c r="C22" s="3">
+      <c r="C22" s="7">
         <v>21.0</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>204</v>
-      </c>
-      <c r="F22" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="G22" s="3" t="s">
-        <v>115</v>
+        <v>202</v>
+      </c>
+      <c r="F22" s="19"/>
+      <c r="G22" s="19" t="s">
+        <v>144</v>
       </c>
       <c r="H22" s="3" t="s">
-        <v>106</v>
+        <v>145</v>
       </c>
       <c r="I22" s="19"/>
-      <c r="J22" s="3" t="s">
-        <v>134</v>
-      </c>
-      <c r="K22" s="3" t="s">
-        <v>135</v>
+      <c r="J22" s="19" t="s">
+        <v>146</v>
+      </c>
+      <c r="K22" s="19" t="s">
+        <v>108</v>
       </c>
       <c r="L22" s="19"/>
       <c r="M22" s="19"/>
       <c r="N22" s="19"/>
       <c r="O22" s="3">
-        <v>0.794</v>
+        <v>0.699</v>
       </c>
       <c r="P22" s="3">
-        <v>0.785</v>
+        <v>0.74</v>
       </c>
       <c r="Q22" s="3">
-        <v>0.907</v>
+        <v>0.812</v>
       </c>
       <c r="R22" s="3">
-        <v>0.926</v>
+        <v>0.859</v>
       </c>
       <c r="S22" s="3">
-        <v>0.925</v>
+        <v>0.863</v>
       </c>
       <c r="T22" s="3">
-        <v>0.925</v>
+        <v>0.819</v>
       </c>
       <c r="U22" s="3">
-        <v>0.922</v>
+        <v>0.838</v>
       </c>
       <c r="V22" s="3">
-        <v>0.935</v>
-      </c>
-      <c r="W22" s="3"/>
+        <v>0.861</v>
+      </c>
+      <c r="W22" s="7">
+        <v>0.862</v>
+      </c>
       <c r="X22" s="3">
-        <v>0.93</v>
+        <v>0.838</v>
       </c>
     </row>
     <row r="23">
@@ -8739,17 +8754,17 @@
       <c r="B23" s="8" t="s">
         <v>171</v>
       </c>
-      <c r="C23" s="8">
+      <c r="C23" s="12">
         <v>22.0</v>
       </c>
       <c r="D23" s="8" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="E23" s="8" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="F23" s="8" t="s">
-        <v>207</v>
+        <v>179</v>
       </c>
       <c r="G23" s="8" t="s">
         <v>115</v>
@@ -8768,32 +8783,34 @@
       <c r="M23" s="21"/>
       <c r="N23" s="21"/>
       <c r="O23" s="8">
-        <v>0.686</v>
+        <v>0.794</v>
       </c>
       <c r="P23" s="8">
-        <v>0.752</v>
+        <v>0.785</v>
       </c>
       <c r="Q23" s="8">
-        <v>0.817</v>
+        <v>0.907</v>
       </c>
       <c r="R23" s="8">
-        <v>0.847</v>
+        <v>0.926</v>
       </c>
       <c r="S23" s="8">
-        <v>0.808</v>
+        <v>0.925</v>
       </c>
       <c r="T23" s="8">
-        <v>0.771</v>
+        <v>0.925</v>
       </c>
       <c r="U23" s="8">
-        <v>0.813</v>
+        <v>0.922</v>
       </c>
       <c r="V23" s="8">
-        <v>0.838</v>
-      </c>
-      <c r="W23" s="8"/>
+        <v>0.935</v>
+      </c>
+      <c r="W23" s="12">
+        <v>0.932</v>
+      </c>
       <c r="X23" s="8">
-        <v>0.788</v>
+        <v>0.93</v>
       </c>
     </row>
     <row r="24">
@@ -8803,17 +8820,17 @@
       <c r="B24" s="3" t="s">
         <v>171</v>
       </c>
-      <c r="C24" s="3">
+      <c r="C24" s="7">
         <v>23.0</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="F24" s="3" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="G24" s="3" t="s">
         <v>115</v>
@@ -8832,32 +8849,34 @@
       <c r="M24" s="19"/>
       <c r="N24" s="19"/>
       <c r="O24" s="3">
-        <v>0.693</v>
+        <v>0.686</v>
       </c>
       <c r="P24" s="3">
-        <v>0.877</v>
+        <v>0.752</v>
       </c>
       <c r="Q24" s="3">
-        <v>0.914</v>
+        <v>0.817</v>
       </c>
       <c r="R24" s="3">
-        <v>0.929</v>
+        <v>0.847</v>
       </c>
       <c r="S24" s="3">
-        <v>0.917</v>
+        <v>0.808</v>
       </c>
       <c r="T24" s="3">
-        <v>0.879</v>
+        <v>0.771</v>
       </c>
       <c r="U24" s="3">
-        <v>0.918</v>
+        <v>0.813</v>
       </c>
       <c r="V24" s="3">
-        <v>0.922</v>
-      </c>
-      <c r="W24" s="3"/>
+        <v>0.838</v>
+      </c>
+      <c r="W24" s="7">
+        <v>0.821</v>
+      </c>
       <c r="X24" s="3">
-        <v>0.902</v>
+        <v>0.788</v>
       </c>
     </row>
     <row r="25">
@@ -8867,59 +8886,63 @@
       <c r="B25" s="8" t="s">
         <v>171</v>
       </c>
-      <c r="C25" s="8">
+      <c r="C25" s="12">
         <v>24.0</v>
       </c>
       <c r="D25" s="8" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="E25" s="8" t="s">
-        <v>212</v>
-      </c>
-      <c r="F25" s="8"/>
+        <v>209</v>
+      </c>
+      <c r="F25" s="8" t="s">
+        <v>210</v>
+      </c>
       <c r="G25" s="8" t="s">
-        <v>105</v>
+        <v>115</v>
       </c>
       <c r="H25" s="8" t="s">
         <v>106</v>
       </c>
       <c r="I25" s="21"/>
       <c r="J25" s="8" t="s">
-        <v>107</v>
+        <v>134</v>
       </c>
       <c r="K25" s="8" t="s">
-        <v>108</v>
+        <v>135</v>
       </c>
       <c r="L25" s="21"/>
       <c r="M25" s="21"/>
       <c r="N25" s="21"/>
       <c r="O25" s="8">
-        <v>0.829</v>
+        <v>0.693</v>
       </c>
       <c r="P25" s="8">
-        <v>0.775</v>
+        <v>0.877</v>
       </c>
       <c r="Q25" s="8">
-        <v>0.837</v>
+        <v>0.914</v>
       </c>
       <c r="R25" s="8">
-        <v>0.89</v>
+        <v>0.929</v>
       </c>
       <c r="S25" s="8">
-        <v>0.876</v>
+        <v>0.917</v>
       </c>
       <c r="T25" s="8">
-        <v>0.868</v>
+        <v>0.879</v>
       </c>
       <c r="U25" s="8">
-        <v>0.861</v>
+        <v>0.918</v>
       </c>
       <c r="V25" s="8">
-        <v>0.858</v>
-      </c>
-      <c r="W25" s="8"/>
+        <v>0.922</v>
+      </c>
+      <c r="W25" s="12">
+        <v>0.928</v>
+      </c>
       <c r="X25" s="8">
-        <v>0.855</v>
+        <v>0.902</v>
       </c>
     </row>
     <row r="26">
@@ -8929,61 +8952,61 @@
       <c r="B26" s="3" t="s">
         <v>171</v>
       </c>
-      <c r="C26" s="3">
+      <c r="C26" s="7">
         <v>25.0</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>214</v>
-      </c>
-      <c r="F26" s="3" t="s">
-        <v>179</v>
-      </c>
+        <v>212</v>
+      </c>
+      <c r="F26" s="3"/>
       <c r="G26" s="3" t="s">
-        <v>115</v>
+        <v>105</v>
       </c>
       <c r="H26" s="3" t="s">
         <v>106</v>
       </c>
       <c r="I26" s="19"/>
       <c r="J26" s="3" t="s">
-        <v>134</v>
+        <v>107</v>
       </c>
       <c r="K26" s="3" t="s">
-        <v>135</v>
+        <v>108</v>
       </c>
       <c r="L26" s="19"/>
       <c r="M26" s="19"/>
       <c r="N26" s="19"/>
       <c r="O26" s="3">
-        <v>0.714</v>
+        <v>0.829</v>
       </c>
       <c r="P26" s="3">
-        <v>0.7</v>
+        <v>0.775</v>
       </c>
       <c r="Q26" s="3">
-        <v>0.797</v>
+        <v>0.837</v>
       </c>
       <c r="R26" s="3">
-        <v>0.842</v>
+        <v>0.89</v>
       </c>
       <c r="S26" s="3">
+        <v>0.876</v>
+      </c>
+      <c r="T26" s="3">
         <v>0.868</v>
       </c>
-      <c r="T26" s="3">
-        <v>0.83</v>
-      </c>
       <c r="U26" s="3">
-        <v>0.851</v>
+        <v>0.861</v>
       </c>
       <c r="V26" s="3">
-        <v>0.863</v>
-      </c>
-      <c r="W26" s="3"/>
+        <v>0.858</v>
+      </c>
+      <c r="W26" s="7">
+        <v>0.895</v>
+      </c>
       <c r="X26" s="3">
-        <v>0.834</v>
+        <v>0.855</v>
       </c>
     </row>
     <row r="27">
@@ -8993,14 +9016,14 @@
       <c r="B27" s="8" t="s">
         <v>171</v>
       </c>
-      <c r="C27" s="8">
+      <c r="C27" s="12">
         <v>26.0</v>
       </c>
       <c r="D27" s="8" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="E27" s="8" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="F27" s="8" t="s">
         <v>179</v>
@@ -9022,32 +9045,34 @@
       <c r="M27" s="21"/>
       <c r="N27" s="21"/>
       <c r="O27" s="8">
-        <v>0.721</v>
+        <v>0.714</v>
       </c>
       <c r="P27" s="8">
-        <v>0.66</v>
+        <v>0.7</v>
       </c>
       <c r="Q27" s="8">
-        <v>0.667</v>
+        <v>0.797</v>
       </c>
       <c r="R27" s="8">
-        <v>0.765</v>
+        <v>0.842</v>
       </c>
       <c r="S27" s="8">
-        <v>0.826</v>
+        <v>0.868</v>
       </c>
       <c r="T27" s="8">
-        <v>0.758</v>
+        <v>0.83</v>
       </c>
       <c r="U27" s="8">
-        <v>0.761</v>
+        <v>0.851</v>
       </c>
       <c r="V27" s="8">
-        <v>0.838</v>
-      </c>
-      <c r="W27" s="8"/>
+        <v>0.863</v>
+      </c>
+      <c r="W27" s="12">
+        <v>0.85</v>
+      </c>
       <c r="X27" s="8">
-        <v>0.818</v>
+        <v>0.834</v>
       </c>
     </row>
     <row r="28">
@@ -9057,14 +9082,14 @@
       <c r="B28" s="3" t="s">
         <v>171</v>
       </c>
-      <c r="C28" s="3">
+      <c r="C28" s="7">
         <v>27.0</v>
       </c>
       <c r="D28" s="3" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="E28" s="3" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="F28" s="3" t="s">
         <v>179</v>
@@ -9086,32 +9111,34 @@
       <c r="M28" s="19"/>
       <c r="N28" s="19"/>
       <c r="O28" s="3">
-        <v>0.714</v>
+        <v>0.721</v>
       </c>
       <c r="P28" s="3">
-        <v>0.815</v>
+        <v>0.66</v>
       </c>
       <c r="Q28" s="3">
-        <v>0.698</v>
+        <v>0.667</v>
       </c>
       <c r="R28" s="3">
-        <v>0.75</v>
+        <v>0.765</v>
       </c>
       <c r="S28" s="3">
-        <v>0.742</v>
+        <v>0.826</v>
       </c>
       <c r="T28" s="3">
-        <v>0.741</v>
+        <v>0.758</v>
       </c>
       <c r="U28" s="3">
-        <v>0.706</v>
+        <v>0.761</v>
       </c>
       <c r="V28" s="3">
-        <v>0.676</v>
-      </c>
-      <c r="W28" s="3"/>
+        <v>0.838</v>
+      </c>
+      <c r="W28" s="7">
+        <v>0.831</v>
+      </c>
       <c r="X28" s="3">
-        <v>0.727</v>
+        <v>0.818</v>
       </c>
     </row>
     <row r="29">
@@ -9121,59 +9148,63 @@
       <c r="B29" s="8" t="s">
         <v>171</v>
       </c>
-      <c r="C29" s="8">
+      <c r="C29" s="12">
         <v>28.0</v>
       </c>
       <c r="D29" s="8" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="E29" s="8" t="s">
-        <v>220</v>
-      </c>
-      <c r="F29" s="8"/>
+        <v>218</v>
+      </c>
+      <c r="F29" s="8" t="s">
+        <v>179</v>
+      </c>
       <c r="G29" s="8" t="s">
-        <v>105</v>
+        <v>115</v>
       </c>
       <c r="H29" s="8" t="s">
         <v>106</v>
       </c>
       <c r="I29" s="21"/>
       <c r="J29" s="8" t="s">
-        <v>107</v>
+        <v>134</v>
       </c>
       <c r="K29" s="8" t="s">
-        <v>108</v>
+        <v>135</v>
       </c>
       <c r="L29" s="21"/>
       <c r="M29" s="21"/>
       <c r="N29" s="21"/>
       <c r="O29" s="8">
-        <v>0.333</v>
+        <v>0.714</v>
       </c>
       <c r="P29" s="8">
-        <v>0.7</v>
+        <v>0.815</v>
       </c>
       <c r="Q29" s="8">
-        <v>0.615</v>
+        <v>0.698</v>
       </c>
       <c r="R29" s="8">
-        <v>0.68</v>
+        <v>0.75</v>
       </c>
       <c r="S29" s="8">
-        <v>0.816</v>
+        <v>0.742</v>
       </c>
       <c r="T29" s="8">
-        <v>0.323</v>
+        <v>0.741</v>
       </c>
       <c r="U29" s="8">
-        <v>0.537</v>
+        <v>0.706</v>
       </c>
       <c r="V29" s="8">
-        <v>0.578</v>
-      </c>
-      <c r="W29" s="8"/>
+        <v>0.676</v>
+      </c>
+      <c r="W29" s="12">
+        <v>0.684</v>
+      </c>
       <c r="X29" s="8">
-        <v>0.714</v>
+        <v>0.727</v>
       </c>
     </row>
     <row r="30">
@@ -9183,14 +9214,14 @@
       <c r="B30" s="3" t="s">
         <v>171</v>
       </c>
-      <c r="C30" s="3">
+      <c r="C30" s="7">
         <v>29.0</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="F30" s="3"/>
       <c r="G30" s="3" t="s">
@@ -9210,32 +9241,34 @@
       <c r="M30" s="19"/>
       <c r="N30" s="19"/>
       <c r="O30" s="3">
-        <v>0.0</v>
+        <v>0.333</v>
       </c>
       <c r="P30" s="3">
-        <v>0.182</v>
+        <v>0.7</v>
       </c>
       <c r="Q30" s="3">
-        <v>0.381</v>
+        <v>0.615</v>
       </c>
       <c r="R30" s="3">
-        <v>0.429</v>
+        <v>0.68</v>
       </c>
       <c r="S30" s="3">
-        <v>0.526</v>
+        <v>0.816</v>
       </c>
       <c r="T30" s="3">
-        <v>0.182</v>
+        <v>0.323</v>
       </c>
       <c r="U30" s="3">
-        <v>0.24</v>
+        <v>0.537</v>
       </c>
       <c r="V30" s="3">
-        <v>0.421</v>
-      </c>
-      <c r="W30" s="3"/>
+        <v>0.578</v>
+      </c>
+      <c r="W30" s="7">
+        <v>0.638</v>
+      </c>
       <c r="X30" s="3">
-        <v>0.387</v>
+        <v>0.714</v>
       </c>
     </row>
     <row r="31">
@@ -9245,61 +9278,61 @@
       <c r="B31" s="8" t="s">
         <v>171</v>
       </c>
-      <c r="C31" s="8">
+      <c r="C31" s="12">
         <v>30.0</v>
       </c>
       <c r="D31" s="8" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="E31" s="8" t="s">
-        <v>224</v>
-      </c>
-      <c r="F31" s="8" t="s">
-        <v>179</v>
-      </c>
+        <v>222</v>
+      </c>
+      <c r="F31" s="8"/>
       <c r="G31" s="8" t="s">
-        <v>115</v>
+        <v>105</v>
       </c>
       <c r="H31" s="8" t="s">
         <v>106</v>
       </c>
       <c r="I31" s="21"/>
       <c r="J31" s="8" t="s">
-        <v>134</v>
+        <v>107</v>
       </c>
       <c r="K31" s="8" t="s">
-        <v>135</v>
+        <v>108</v>
       </c>
       <c r="L31" s="21"/>
       <c r="M31" s="21"/>
       <c r="N31" s="21"/>
       <c r="O31" s="8">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="P31" s="8">
-        <v>0.0</v>
+        <v>0.182</v>
       </c>
       <c r="Q31" s="8">
-        <v>0.667</v>
+        <v>0.381</v>
       </c>
       <c r="R31" s="8">
-        <v>0.8</v>
+        <v>0.429</v>
       </c>
       <c r="S31" s="8">
-        <v>0.8</v>
+        <v>0.526</v>
       </c>
       <c r="T31" s="8">
-        <v>0.8</v>
+        <v>0.182</v>
       </c>
       <c r="U31" s="8">
-        <v>0.6</v>
+        <v>0.24</v>
       </c>
       <c r="V31" s="8">
-        <v>0.6</v>
-      </c>
-      <c r="W31" s="8"/>
+        <v>0.421</v>
+      </c>
+      <c r="W31" s="12">
+        <v>0.579</v>
+      </c>
       <c r="X31" s="8">
-        <v>0.667</v>
+        <v>0.387</v>
       </c>
     </row>
     <row r="32">
@@ -9309,14 +9342,14 @@
       <c r="B32" s="3" t="s">
         <v>171</v>
       </c>
-      <c r="C32" s="3">
+      <c r="C32" s="7">
         <v>31.0</v>
       </c>
       <c r="D32" s="3" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="E32" s="3" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="F32" s="3" t="s">
         <v>179</v>
@@ -9338,32 +9371,34 @@
       <c r="M32" s="19"/>
       <c r="N32" s="19"/>
       <c r="O32" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="P32" s="3">
         <v>0.0</v>
       </c>
-      <c r="P32" s="3">
-        <v>0.286</v>
-      </c>
       <c r="Q32" s="3">
-        <v>0.488</v>
+        <v>0.667</v>
       </c>
       <c r="R32" s="3">
-        <v>0.507</v>
+        <v>0.8</v>
       </c>
       <c r="S32" s="3">
-        <v>0.75</v>
+        <v>0.8</v>
       </c>
       <c r="T32" s="3">
-        <v>0.75</v>
+        <v>0.8</v>
       </c>
       <c r="U32" s="3">
+        <v>0.6</v>
+      </c>
+      <c r="V32" s="3">
+        <v>0.6</v>
+      </c>
+      <c r="W32" s="7">
+        <v>0.769</v>
+      </c>
+      <c r="X32" s="3">
         <v>0.667</v>
-      </c>
-      <c r="V32" s="3">
-        <v>0.571</v>
-      </c>
-      <c r="W32" s="3"/>
-      <c r="X32" s="3">
-        <v>0.571</v>
       </c>
     </row>
     <row r="33">
@@ -9373,17 +9408,17 @@
       <c r="B33" s="8" t="s">
         <v>171</v>
       </c>
-      <c r="C33" s="8">
+      <c r="C33" s="12">
         <v>32.0</v>
       </c>
       <c r="D33" s="8" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="E33" s="8" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="F33" s="8" t="s">
-        <v>229</v>
+        <v>179</v>
       </c>
       <c r="G33" s="8" t="s">
         <v>115</v>
@@ -9401,31 +9436,35 @@
       <c r="L33" s="21"/>
       <c r="M33" s="21"/>
       <c r="N33" s="21"/>
-      <c r="O33" s="8"/>
+      <c r="O33" s="8">
+        <v>0.0</v>
+      </c>
       <c r="P33" s="8">
+        <v>0.286</v>
+      </c>
+      <c r="Q33" s="8">
+        <v>0.488</v>
+      </c>
+      <c r="R33" s="8">
+        <v>0.507</v>
+      </c>
+      <c r="S33" s="8">
+        <v>0.75</v>
+      </c>
+      <c r="T33" s="8">
+        <v>0.75</v>
+      </c>
+      <c r="U33" s="8">
         <v>0.667</v>
       </c>
-      <c r="Q33" s="8">
-        <v>0.667</v>
-      </c>
-      <c r="R33" s="8">
-        <v>0.96</v>
-      </c>
-      <c r="S33" s="8">
-        <v>0.977</v>
-      </c>
-      <c r="T33" s="8">
-        <v>0.737</v>
-      </c>
-      <c r="U33" s="8">
-        <v>0.85</v>
-      </c>
       <c r="V33" s="8">
-        <v>0.9</v>
-      </c>
-      <c r="W33" s="8"/>
+        <v>0.571</v>
+      </c>
+      <c r="W33" s="12">
+        <v>0.8</v>
+      </c>
       <c r="X33" s="8">
-        <v>0.741</v>
+        <v>0.571</v>
       </c>
     </row>
     <row r="34">
@@ -9435,57 +9474,61 @@
       <c r="B34" s="3" t="s">
         <v>171</v>
       </c>
-      <c r="C34" s="3">
+      <c r="C34" s="7">
         <v>33.0</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="E34" s="3" t="s">
-        <v>231</v>
-      </c>
-      <c r="F34" s="3"/>
+        <v>228</v>
+      </c>
+      <c r="F34" s="3" t="s">
+        <v>229</v>
+      </c>
       <c r="G34" s="3" t="s">
         <v>115</v>
       </c>
       <c r="H34" s="3" t="s">
         <v>106</v>
       </c>
-      <c r="I34" s="3"/>
+      <c r="I34" s="19"/>
       <c r="J34" s="3" t="s">
-        <v>121</v>
+        <v>134</v>
       </c>
       <c r="K34" s="3" t="s">
-        <v>116</v>
-      </c>
-      <c r="L34" s="3"/>
-      <c r="M34" s="3"/>
+        <v>135</v>
+      </c>
+      <c r="L34" s="19"/>
+      <c r="M34" s="19"/>
       <c r="N34" s="19"/>
-      <c r="O34" s="19"/>
+      <c r="O34" s="3"/>
       <c r="P34" s="3">
-        <v>0.0</v>
+        <v>0.667</v>
       </c>
       <c r="Q34" s="3">
-        <v>0.0</v>
+        <v>0.667</v>
       </c>
       <c r="R34" s="3">
-        <v>0.579</v>
+        <v>0.96</v>
       </c>
       <c r="S34" s="3">
-        <v>0.759</v>
+        <v>0.977</v>
       </c>
       <c r="T34" s="3">
-        <v>0.72</v>
+        <v>0.737</v>
       </c>
       <c r="U34" s="3">
-        <v>0.696</v>
+        <v>0.85</v>
       </c>
       <c r="V34" s="3">
-        <v>0.786</v>
-      </c>
-      <c r="W34" s="3"/>
+        <v>0.9</v>
+      </c>
+      <c r="W34" s="7">
+        <v>0.905</v>
+      </c>
       <c r="X34" s="3">
-        <v>0.667</v>
+        <v>0.741</v>
       </c>
     </row>
     <row r="35">
@@ -9495,59 +9538,59 @@
       <c r="B35" s="8" t="s">
         <v>171</v>
       </c>
-      <c r="C35" s="8">
+      <c r="C35" s="12">
         <v>34.0</v>
       </c>
       <c r="D35" s="8" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="E35" s="8" t="s">
-        <v>233</v>
-      </c>
-      <c r="F35" s="8" t="s">
-        <v>179</v>
-      </c>
+        <v>231</v>
+      </c>
+      <c r="F35" s="8"/>
       <c r="G35" s="8" t="s">
         <v>115</v>
       </c>
       <c r="H35" s="8" t="s">
         <v>106</v>
       </c>
-      <c r="I35" s="21"/>
+      <c r="I35" s="8"/>
       <c r="J35" s="8" t="s">
-        <v>134</v>
+        <v>121</v>
       </c>
       <c r="K35" s="8" t="s">
-        <v>135</v>
-      </c>
-      <c r="L35" s="21"/>
-      <c r="M35" s="21"/>
+        <v>116</v>
+      </c>
+      <c r="L35" s="8"/>
+      <c r="M35" s="8"/>
       <c r="N35" s="21"/>
       <c r="O35" s="21"/>
       <c r="P35" s="8">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="Q35" s="8">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="R35" s="8">
+        <v>0.579</v>
+      </c>
+      <c r="S35" s="8">
+        <v>0.759</v>
+      </c>
+      <c r="T35" s="8">
+        <v>0.72</v>
+      </c>
+      <c r="U35" s="8">
+        <v>0.696</v>
+      </c>
+      <c r="V35" s="8">
+        <v>0.786</v>
+      </c>
+      <c r="W35" s="12">
+        <v>0.786</v>
+      </c>
+      <c r="X35" s="8">
         <v>0.667</v>
-      </c>
-      <c r="S35" s="8">
-        <v>0.667</v>
-      </c>
-      <c r="T35" s="8">
-        <v>0.714</v>
-      </c>
-      <c r="U35" s="8">
-        <v>0.714</v>
-      </c>
-      <c r="V35" s="8">
-        <v>0.927</v>
-      </c>
-      <c r="W35" s="8"/>
-      <c r="X35" s="8">
-        <v>0.927</v>
       </c>
     </row>
     <row r="36">
@@ -9557,14 +9600,14 @@
       <c r="B36" s="3" t="s">
         <v>171</v>
       </c>
-      <c r="C36" s="3">
+      <c r="C36" s="7">
         <v>35.0</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="E36" s="3" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="F36" s="3" t="s">
         <v>179</v>
@@ -9587,13 +9630,13 @@
       <c r="N36" s="19"/>
       <c r="O36" s="19"/>
       <c r="P36" s="3">
-        <v>0.25</v>
+        <v>1.0</v>
       </c>
       <c r="Q36" s="3">
-        <v>0.545</v>
+        <v>1.0</v>
       </c>
       <c r="R36" s="3">
-        <v>0.467</v>
+        <v>0.667</v>
       </c>
       <c r="S36" s="3">
         <v>0.667</v>
@@ -9605,11 +9648,13 @@
         <v>0.714</v>
       </c>
       <c r="V36" s="3">
-        <v>0.905</v>
-      </c>
-      <c r="W36" s="3"/>
+        <v>0.927</v>
+      </c>
+      <c r="W36" s="7">
+        <v>0.913</v>
+      </c>
       <c r="X36" s="3">
-        <v>0.905</v>
+        <v>0.927</v>
       </c>
     </row>
     <row r="37">
@@ -9619,14 +9664,14 @@
       <c r="B37" s="8" t="s">
         <v>171</v>
       </c>
-      <c r="C37" s="8">
+      <c r="C37" s="12">
         <v>36.0</v>
       </c>
       <c r="D37" s="8" t="s">
-        <v>132</v>
+        <v>234</v>
       </c>
       <c r="E37" s="8" t="s">
-        <v>133</v>
+        <v>235</v>
       </c>
       <c r="F37" s="8" t="s">
         <v>179</v>
@@ -9637,43 +9682,43 @@
       <c r="H37" s="8" t="s">
         <v>106</v>
       </c>
-      <c r="I37" s="8"/>
+      <c r="I37" s="21"/>
       <c r="J37" s="8" t="s">
         <v>134</v>
       </c>
       <c r="K37" s="8" t="s">
         <v>135</v>
       </c>
-      <c r="L37" s="8"/>
-      <c r="M37" s="8"/>
+      <c r="L37" s="21"/>
+      <c r="M37" s="21"/>
       <c r="N37" s="21"/>
-      <c r="O37" s="8">
-        <v>0.8</v>
-      </c>
+      <c r="O37" s="21"/>
       <c r="P37" s="8">
-        <v>0.826</v>
+        <v>0.25</v>
       </c>
       <c r="Q37" s="8">
-        <v>0.851</v>
+        <v>0.545</v>
       </c>
       <c r="R37" s="8">
-        <v>0.887</v>
+        <v>0.467</v>
       </c>
       <c r="S37" s="8">
-        <v>0.778</v>
+        <v>0.667</v>
       </c>
       <c r="T37" s="8">
         <v>0.714</v>
       </c>
       <c r="U37" s="8">
-        <v>0.8</v>
+        <v>0.714</v>
       </c>
       <c r="V37" s="8">
-        <v>0.8</v>
-      </c>
-      <c r="W37" s="8"/>
+        <v>0.905</v>
+      </c>
+      <c r="W37" s="12">
+        <v>0.905</v>
+      </c>
       <c r="X37" s="8">
-        <v>0.857</v>
+        <v>0.905</v>
       </c>
     </row>
     <row r="38">
@@ -9683,40 +9728,64 @@
       <c r="B38" s="3" t="s">
         <v>171</v>
       </c>
-      <c r="C38" s="3">
+      <c r="C38" s="7">
         <v>37.0</v>
       </c>
       <c r="D38" s="3" t="s">
-        <v>236</v>
-      </c>
-      <c r="E38" s="19"/>
-      <c r="F38" s="19"/>
-      <c r="G38" s="7" t="s">
-        <v>144</v>
+        <v>132</v>
+      </c>
+      <c r="E38" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="F38" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="G38" s="3" t="s">
+        <v>115</v>
       </c>
       <c r="H38" s="3" t="s">
-        <v>145</v>
-      </c>
-      <c r="I38" s="19"/>
+        <v>106</v>
+      </c>
+      <c r="I38" s="3"/>
       <c r="J38" s="3" t="s">
-        <v>146</v>
-      </c>
-      <c r="K38" s="7" t="s">
-        <v>108</v>
-      </c>
-      <c r="L38" s="19"/>
-      <c r="M38" s="19"/>
+        <v>134</v>
+      </c>
+      <c r="K38" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="L38" s="3"/>
+      <c r="M38" s="3"/>
       <c r="N38" s="19"/>
-      <c r="O38" s="19"/>
-      <c r="P38" s="19"/>
-      <c r="Q38" s="19"/>
-      <c r="R38" s="19"/>
-      <c r="S38" s="19"/>
-      <c r="T38" s="19"/>
-      <c r="U38" s="19"/>
-      <c r="V38" s="19"/>
-      <c r="W38" s="19"/>
-      <c r="X38" s="19"/>
+      <c r="O38" s="3">
+        <v>0.8</v>
+      </c>
+      <c r="P38" s="3">
+        <v>0.826</v>
+      </c>
+      <c r="Q38" s="3">
+        <v>0.851</v>
+      </c>
+      <c r="R38" s="3">
+        <v>0.887</v>
+      </c>
+      <c r="S38" s="3">
+        <v>0.778</v>
+      </c>
+      <c r="T38" s="3">
+        <v>0.714</v>
+      </c>
+      <c r="U38" s="3">
+        <v>0.8</v>
+      </c>
+      <c r="V38" s="3">
+        <v>0.8</v>
+      </c>
+      <c r="W38" s="7">
+        <v>0.849</v>
+      </c>
+      <c r="X38" s="3">
+        <v>0.857</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="8" t="s">
@@ -9725,28 +9794,26 @@
       <c r="B39" s="8" t="s">
         <v>171</v>
       </c>
-      <c r="C39" s="8">
+      <c r="C39" s="12">
         <v>38.0</v>
       </c>
       <c r="D39" s="8" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="E39" s="21"/>
-      <c r="F39" s="8" t="s">
-        <v>179</v>
-      </c>
-      <c r="G39" s="8" t="s">
-        <v>200</v>
+      <c r="F39" s="21"/>
+      <c r="G39" s="12" t="s">
+        <v>144</v>
       </c>
       <c r="H39" s="8" t="s">
-        <v>106</v>
+        <v>145</v>
       </c>
       <c r="I39" s="21"/>
       <c r="J39" s="8" t="s">
-        <v>134</v>
-      </c>
-      <c r="K39" s="8" t="s">
-        <v>135</v>
+        <v>146</v>
+      </c>
+      <c r="K39" s="12" t="s">
+        <v>108</v>
       </c>
       <c r="L39" s="21"/>
       <c r="M39" s="21"/>
@@ -9759,7 +9826,9 @@
       <c r="T39" s="21"/>
       <c r="U39" s="21"/>
       <c r="V39" s="21"/>
-      <c r="W39" s="21"/>
+      <c r="W39" s="12">
+        <v>0.983</v>
+      </c>
       <c r="X39" s="21"/>
     </row>
     <row r="40">
@@ -9769,11 +9838,11 @@
       <c r="B40" s="3" t="s">
         <v>171</v>
       </c>
-      <c r="C40" s="3">
+      <c r="C40" s="7">
         <v>39.0</v>
       </c>
       <c r="D40" s="3" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="E40" s="19"/>
       <c r="F40" s="3" t="s">
@@ -9803,7 +9872,9 @@
       <c r="T40" s="19"/>
       <c r="U40" s="19"/>
       <c r="V40" s="19"/>
-      <c r="W40" s="19"/>
+      <c r="W40" s="7">
+        <v>0.947</v>
+      </c>
       <c r="X40" s="19"/>
     </row>
     <row r="41">
@@ -9813,14 +9884,16 @@
       <c r="B41" s="8" t="s">
         <v>171</v>
       </c>
-      <c r="C41" s="8">
+      <c r="C41" s="12">
         <v>40.0</v>
       </c>
       <c r="D41" s="8" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="E41" s="21"/>
-      <c r="F41" s="21"/>
+      <c r="F41" s="8" t="s">
+        <v>179</v>
+      </c>
       <c r="G41" s="8" t="s">
         <v>200</v>
       </c>
@@ -9829,10 +9902,10 @@
       </c>
       <c r="I41" s="21"/>
       <c r="J41" s="8" t="s">
-        <v>121</v>
-      </c>
-      <c r="K41" s="12" t="s">
-        <v>116</v>
+        <v>134</v>
+      </c>
+      <c r="K41" s="8" t="s">
+        <v>135</v>
       </c>
       <c r="L41" s="21"/>
       <c r="M41" s="21"/>
@@ -9845,7 +9918,9 @@
       <c r="T41" s="21"/>
       <c r="U41" s="21"/>
       <c r="V41" s="21"/>
-      <c r="W41" s="21"/>
+      <c r="W41" s="12">
+        <v>1.0</v>
+      </c>
       <c r="X41" s="21"/>
     </row>
     <row r="42">
@@ -9855,11 +9930,11 @@
       <c r="B42" s="3" t="s">
         <v>171</v>
       </c>
-      <c r="C42" s="3">
+      <c r="C42" s="7">
         <v>41.0</v>
       </c>
       <c r="D42" s="3" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="E42" s="19"/>
       <c r="F42" s="19"/>
@@ -9871,10 +9946,10 @@
       </c>
       <c r="I42" s="19"/>
       <c r="J42" s="3" t="s">
-        <v>107</v>
+        <v>121</v>
       </c>
       <c r="K42" s="7" t="s">
-        <v>108</v>
+        <v>116</v>
       </c>
       <c r="L42" s="19"/>
       <c r="M42" s="19"/>
@@ -9887,7 +9962,9 @@
       <c r="T42" s="19"/>
       <c r="U42" s="19"/>
       <c r="V42" s="19"/>
-      <c r="W42" s="19"/>
+      <c r="W42" s="7">
+        <v>1.0</v>
+      </c>
       <c r="X42" s="19"/>
     </row>
     <row r="43">
@@ -9897,11 +9974,11 @@
       <c r="B43" s="8" t="s">
         <v>171</v>
       </c>
-      <c r="C43" s="8">
+      <c r="C43" s="12">
         <v>42.0</v>
       </c>
       <c r="D43" s="8" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="E43" s="21"/>
       <c r="F43" s="21"/>
@@ -9929,7 +10006,9 @@
       <c r="T43" s="21"/>
       <c r="U43" s="21"/>
       <c r="V43" s="21"/>
-      <c r="W43" s="21"/>
+      <c r="W43" s="12">
+        <v>1.0</v>
+      </c>
       <c r="X43" s="21"/>
     </row>
     <row r="44">
@@ -9939,16 +10018,14 @@
       <c r="B44" s="3" t="s">
         <v>171</v>
       </c>
-      <c r="C44" s="3">
+      <c r="C44" s="7">
         <v>43.0</v>
       </c>
       <c r="D44" s="3" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="E44" s="19"/>
-      <c r="F44" s="3" t="s">
-        <v>243</v>
-      </c>
+      <c r="F44" s="19"/>
       <c r="G44" s="3" t="s">
         <v>200</v>
       </c>
@@ -9957,10 +10034,10 @@
       </c>
       <c r="I44" s="19"/>
       <c r="J44" s="3" t="s">
-        <v>121</v>
+        <v>107</v>
       </c>
       <c r="K44" s="7" t="s">
-        <v>116</v>
+        <v>108</v>
       </c>
       <c r="L44" s="19"/>
       <c r="M44" s="19"/>
@@ -9973,7 +10050,9 @@
       <c r="T44" s="19"/>
       <c r="U44" s="19"/>
       <c r="V44" s="19"/>
-      <c r="W44" s="19"/>
+      <c r="W44" s="7">
+        <v>0.667</v>
+      </c>
       <c r="X44" s="19"/>
     </row>
     <row r="45">
@@ -9983,15 +10062,15 @@
       <c r="B45" s="8" t="s">
         <v>171</v>
       </c>
-      <c r="C45" s="8">
+      <c r="C45" s="12">
         <v>44.0</v>
       </c>
       <c r="D45" s="8" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="E45" s="21"/>
       <c r="F45" s="8" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="G45" s="8" t="s">
         <v>200</v>
@@ -10001,10 +10080,10 @@
       </c>
       <c r="I45" s="21"/>
       <c r="J45" s="8" t="s">
-        <v>134</v>
+        <v>121</v>
       </c>
       <c r="K45" s="12" t="s">
-        <v>135</v>
+        <v>116</v>
       </c>
       <c r="L45" s="21"/>
       <c r="M45" s="21"/>
@@ -10017,7 +10096,9 @@
       <c r="T45" s="21"/>
       <c r="U45" s="21"/>
       <c r="V45" s="21"/>
-      <c r="W45" s="21"/>
+      <c r="W45" s="12">
+        <v>0.889</v>
+      </c>
       <c r="X45" s="21"/>
     </row>
     <row r="46">
@@ -10027,15 +10108,15 @@
       <c r="B46" s="3" t="s">
         <v>171</v>
       </c>
-      <c r="C46" s="3">
+      <c r="C46" s="7">
         <v>45.0</v>
       </c>
       <c r="D46" s="3" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="E46" s="19"/>
       <c r="F46" s="3" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="G46" s="3" t="s">
         <v>200</v>
@@ -10061,7 +10142,9 @@
       <c r="T46" s="19"/>
       <c r="U46" s="19"/>
       <c r="V46" s="19"/>
-      <c r="W46" s="19"/>
+      <c r="W46" s="7">
+        <v>0.921</v>
+      </c>
       <c r="X46" s="19"/>
     </row>
     <row r="47">
@@ -10071,15 +10154,15 @@
       <c r="B47" s="8" t="s">
         <v>171</v>
       </c>
-      <c r="C47" s="8">
+      <c r="C47" s="12">
         <v>46.0</v>
       </c>
       <c r="D47" s="8" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="E47" s="21"/>
       <c r="F47" s="8" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="G47" s="8" t="s">
         <v>200</v>
@@ -10105,7 +10188,9 @@
       <c r="T47" s="21"/>
       <c r="U47" s="21"/>
       <c r="V47" s="21"/>
-      <c r="W47" s="21"/>
+      <c r="W47" s="12">
+        <v>0.857</v>
+      </c>
       <c r="X47" s="21"/>
     </row>
     <row r="48">
@@ -10115,28 +10200,28 @@
       <c r="B48" s="3" t="s">
         <v>171</v>
       </c>
-      <c r="C48" s="3">
+      <c r="C48" s="7">
         <v>47.0</v>
       </c>
       <c r="D48" s="3" t="s">
-        <v>249</v>
-      </c>
-      <c r="E48" s="3" t="s">
-        <v>250</v>
-      </c>
-      <c r="F48" s="19"/>
+        <v>248</v>
+      </c>
+      <c r="E48" s="19"/>
+      <c r="F48" s="3" t="s">
+        <v>245</v>
+      </c>
       <c r="G48" s="3" t="s">
-        <v>144</v>
+        <v>200</v>
       </c>
       <c r="H48" s="3" t="s">
-        <v>145</v>
+        <v>106</v>
       </c>
       <c r="I48" s="19"/>
       <c r="J48" s="3" t="s">
-        <v>146</v>
+        <v>134</v>
       </c>
       <c r="K48" s="7" t="s">
-        <v>108</v>
+        <v>135</v>
       </c>
       <c r="L48" s="19"/>
       <c r="M48" s="19"/>
@@ -10149,7 +10234,9 @@
       <c r="T48" s="19"/>
       <c r="U48" s="19"/>
       <c r="V48" s="19"/>
-      <c r="W48" s="19"/>
+      <c r="W48" s="7">
+        <v>0.857</v>
+      </c>
       <c r="X48" s="19"/>
     </row>
     <row r="49">
@@ -10159,30 +10246,28 @@
       <c r="B49" s="8" t="s">
         <v>171</v>
       </c>
-      <c r="C49" s="8">
+      <c r="C49" s="12">
         <v>48.0</v>
       </c>
       <c r="D49" s="8" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="E49" s="8" t="s">
-        <v>252</v>
-      </c>
-      <c r="F49" s="8" t="s">
-        <v>179</v>
-      </c>
+        <v>250</v>
+      </c>
+      <c r="F49" s="21"/>
       <c r="G49" s="8" t="s">
-        <v>200</v>
+        <v>144</v>
       </c>
       <c r="H49" s="8" t="s">
-        <v>106</v>
+        <v>145</v>
       </c>
       <c r="I49" s="21"/>
       <c r="J49" s="8" t="s">
-        <v>134</v>
+        <v>146</v>
       </c>
       <c r="K49" s="12" t="s">
-        <v>135</v>
+        <v>108</v>
       </c>
       <c r="L49" s="21"/>
       <c r="M49" s="21"/>
@@ -10195,7 +10280,9 @@
       <c r="T49" s="21"/>
       <c r="U49" s="21"/>
       <c r="V49" s="21"/>
-      <c r="W49" s="21"/>
+      <c r="W49" s="12">
+        <v>0.969</v>
+      </c>
       <c r="X49" s="21"/>
     </row>
     <row r="50">
@@ -10205,14 +10292,14 @@
       <c r="B50" s="3" t="s">
         <v>171</v>
       </c>
-      <c r="C50" s="3">
+      <c r="C50" s="7">
         <v>49.0</v>
       </c>
       <c r="D50" s="3" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="E50" s="3" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="F50" s="3" t="s">
         <v>179</v>
@@ -10241,7 +10328,9 @@
       <c r="T50" s="19"/>
       <c r="U50" s="19"/>
       <c r="V50" s="19"/>
-      <c r="W50" s="19"/>
+      <c r="W50" s="7">
+        <v>0.938</v>
+      </c>
       <c r="X50" s="19"/>
     </row>
     <row r="51">
@@ -10251,16 +10340,18 @@
       <c r="B51" s="8" t="s">
         <v>171</v>
       </c>
-      <c r="C51" s="8">
+      <c r="C51" s="12">
         <v>50.0</v>
       </c>
       <c r="D51" s="8" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="E51" s="8" t="s">
-        <v>256</v>
-      </c>
-      <c r="F51" s="21"/>
+        <v>254</v>
+      </c>
+      <c r="F51" s="8" t="s">
+        <v>179</v>
+      </c>
       <c r="G51" s="8" t="s">
         <v>200</v>
       </c>
@@ -10269,10 +10360,10 @@
       </c>
       <c r="I51" s="21"/>
       <c r="J51" s="8" t="s">
-        <v>107</v>
+        <v>134</v>
       </c>
       <c r="K51" s="12" t="s">
-        <v>108</v>
+        <v>135</v>
       </c>
       <c r="L51" s="21"/>
       <c r="M51" s="21"/>
@@ -10285,7 +10376,9 @@
       <c r="T51" s="21"/>
       <c r="U51" s="21"/>
       <c r="V51" s="21"/>
-      <c r="W51" s="21"/>
+      <c r="W51" s="12">
+        <v>1.0</v>
+      </c>
       <c r="X51" s="21"/>
     </row>
     <row r="52">
@@ -10295,13 +10388,15 @@
       <c r="B52" s="3" t="s">
         <v>171</v>
       </c>
-      <c r="C52" s="3">
+      <c r="C52" s="7">
         <v>51.0</v>
       </c>
       <c r="D52" s="3" t="s">
-        <v>257</v>
-      </c>
-      <c r="E52" s="19"/>
+        <v>255</v>
+      </c>
+      <c r="E52" s="3" t="s">
+        <v>256</v>
+      </c>
       <c r="F52" s="19"/>
       <c r="G52" s="3" t="s">
         <v>200</v>
@@ -10327,7 +10422,9 @@
       <c r="T52" s="19"/>
       <c r="U52" s="19"/>
       <c r="V52" s="19"/>
-      <c r="W52" s="19"/>
+      <c r="W52" s="7">
+        <v>0.889</v>
+      </c>
       <c r="X52" s="19"/>
     </row>
     <row r="53">
@@ -10337,28 +10434,26 @@
       <c r="B53" s="8" t="s">
         <v>171</v>
       </c>
-      <c r="C53" s="8">
+      <c r="C53" s="12">
         <v>52.0</v>
       </c>
       <c r="D53" s="8" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="E53" s="21"/>
-      <c r="F53" s="8" t="s">
-        <v>245</v>
-      </c>
-      <c r="G53" s="12" t="s">
-        <v>105</v>
+      <c r="F53" s="21"/>
+      <c r="G53" s="8" t="s">
+        <v>200</v>
       </c>
       <c r="H53" s="8" t="s">
         <v>106</v>
       </c>
       <c r="I53" s="21"/>
       <c r="J53" s="8" t="s">
-        <v>134</v>
+        <v>107</v>
       </c>
       <c r="K53" s="12" t="s">
-        <v>135</v>
+        <v>108</v>
       </c>
       <c r="L53" s="21"/>
       <c r="M53" s="21"/>
@@ -10371,7 +10466,9 @@
       <c r="T53" s="21"/>
       <c r="U53" s="21"/>
       <c r="V53" s="21"/>
-      <c r="W53" s="21"/>
+      <c r="W53" s="12">
+        <v>0.991</v>
+      </c>
       <c r="X53" s="21"/>
     </row>
     <row r="54">
@@ -10381,28 +10478,28 @@
       <c r="B54" s="3" t="s">
         <v>171</v>
       </c>
-      <c r="C54" s="3">
+      <c r="C54" s="7">
         <v>53.0</v>
       </c>
       <c r="D54" s="3" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="E54" s="19"/>
       <c r="F54" s="3" t="s">
-        <v>243</v>
-      </c>
-      <c r="G54" s="3" t="s">
-        <v>200</v>
+        <v>245</v>
+      </c>
+      <c r="G54" s="7" t="s">
+        <v>105</v>
       </c>
       <c r="H54" s="3" t="s">
         <v>106</v>
       </c>
       <c r="I54" s="19"/>
       <c r="J54" s="3" t="s">
-        <v>121</v>
+        <v>134</v>
       </c>
       <c r="K54" s="7" t="s">
-        <v>116</v>
+        <v>135</v>
       </c>
       <c r="L54" s="19"/>
       <c r="M54" s="19"/>
@@ -10415,7 +10512,9 @@
       <c r="T54" s="19"/>
       <c r="U54" s="19"/>
       <c r="V54" s="19"/>
-      <c r="W54" s="19"/>
+      <c r="W54" s="7">
+        <v>0.88</v>
+      </c>
       <c r="X54" s="19"/>
     </row>
     <row r="55">
@@ -10425,15 +10524,15 @@
       <c r="B55" s="8" t="s">
         <v>171</v>
       </c>
-      <c r="C55" s="8">
+      <c r="C55" s="12">
         <v>54.0</v>
       </c>
       <c r="D55" s="8" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="E55" s="21"/>
       <c r="F55" s="8" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="G55" s="8" t="s">
         <v>200</v>
@@ -10443,10 +10542,10 @@
       </c>
       <c r="I55" s="21"/>
       <c r="J55" s="8" t="s">
-        <v>134</v>
+        <v>121</v>
       </c>
       <c r="K55" s="12" t="s">
-        <v>135</v>
+        <v>116</v>
       </c>
       <c r="L55" s="21"/>
       <c r="M55" s="21"/>
@@ -10459,7 +10558,9 @@
       <c r="T55" s="21"/>
       <c r="U55" s="21"/>
       <c r="V55" s="21"/>
-      <c r="W55" s="21"/>
+      <c r="W55" s="12">
+        <v>0.933</v>
+      </c>
       <c r="X55" s="21"/>
     </row>
     <row r="56">
@@ -10469,11 +10570,11 @@
       <c r="B56" s="3" t="s">
         <v>171</v>
       </c>
-      <c r="C56" s="3">
+      <c r="C56" s="7">
         <v>55.0</v>
       </c>
       <c r="D56" s="3" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="E56" s="19"/>
       <c r="F56" s="3" t="s">
@@ -10503,7 +10604,9 @@
       <c r="T56" s="19"/>
       <c r="U56" s="19"/>
       <c r="V56" s="19"/>
-      <c r="W56" s="19"/>
+      <c r="W56" s="7">
+        <v>0.881</v>
+      </c>
       <c r="X56" s="19"/>
     </row>
     <row r="57">
@@ -10513,11 +10616,11 @@
       <c r="B57" s="8" t="s">
         <v>171</v>
       </c>
-      <c r="C57" s="8">
+      <c r="C57" s="12">
         <v>56.0</v>
       </c>
       <c r="D57" s="8" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="E57" s="21"/>
       <c r="F57" s="8" t="s">
@@ -10547,7 +10650,9 @@
       <c r="T57" s="21"/>
       <c r="U57" s="21"/>
       <c r="V57" s="21"/>
-      <c r="W57" s="21"/>
+      <c r="W57" s="12">
+        <v>1.0</v>
+      </c>
       <c r="X57" s="21"/>
     </row>
     <row r="58">
@@ -10557,15 +10662,15 @@
       <c r="B58" s="3" t="s">
         <v>171</v>
       </c>
-      <c r="C58" s="3">
+      <c r="C58" s="7">
         <v>57.0</v>
       </c>
       <c r="D58" s="3" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="E58" s="19"/>
       <c r="F58" s="3" t="s">
-        <v>179</v>
+        <v>245</v>
       </c>
       <c r="G58" s="3" t="s">
         <v>200</v>
@@ -10591,7 +10696,9 @@
       <c r="T58" s="19"/>
       <c r="U58" s="19"/>
       <c r="V58" s="19"/>
-      <c r="W58" s="19"/>
+      <c r="W58" s="7">
+        <v>0.833</v>
+      </c>
       <c r="X58" s="19"/>
     </row>
     <row r="59">
@@ -10601,11 +10708,11 @@
       <c r="B59" s="8" t="s">
         <v>171</v>
       </c>
-      <c r="C59" s="8">
+      <c r="C59" s="12">
         <v>58.0</v>
       </c>
       <c r="D59" s="8" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="E59" s="21"/>
       <c r="F59" s="8" t="s">
@@ -10635,7 +10742,9 @@
       <c r="T59" s="21"/>
       <c r="U59" s="21"/>
       <c r="V59" s="21"/>
-      <c r="W59" s="21"/>
+      <c r="W59" s="12">
+        <v>0.716</v>
+      </c>
       <c r="X59" s="21"/>
     </row>
     <row r="60">
@@ -10645,14 +10754,16 @@
       <c r="B60" s="3" t="s">
         <v>171</v>
       </c>
-      <c r="C60" s="3">
+      <c r="C60" s="7">
         <v>59.0</v>
       </c>
       <c r="D60" s="3" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="E60" s="19"/>
-      <c r="F60" s="19"/>
+      <c r="F60" s="3" t="s">
+        <v>179</v>
+      </c>
       <c r="G60" s="3" t="s">
         <v>200</v>
       </c>
@@ -10677,7 +10788,9 @@
       <c r="T60" s="19"/>
       <c r="U60" s="19"/>
       <c r="V60" s="19"/>
-      <c r="W60" s="19"/>
+      <c r="W60" s="7">
+        <v>0.742</v>
+      </c>
       <c r="X60" s="19"/>
     </row>
     <row r="61">
@@ -10691,7 +10804,7 @@
         <v>60.0</v>
       </c>
       <c r="D61" s="8" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="E61" s="21"/>
       <c r="F61" s="21"/>
@@ -10702,7 +10815,7 @@
         <v>106</v>
       </c>
       <c r="I61" s="21"/>
-      <c r="J61" s="12" t="s">
+      <c r="J61" s="8" t="s">
         <v>134</v>
       </c>
       <c r="K61" s="12" t="s">
@@ -10719,7 +10832,9 @@
       <c r="T61" s="21"/>
       <c r="U61" s="21"/>
       <c r="V61" s="21"/>
-      <c r="W61" s="21"/>
+      <c r="W61" s="12">
+        <v>0.818</v>
+      </c>
       <c r="X61" s="21"/>
     </row>
     <row r="62">
@@ -10733,7 +10848,7 @@
         <v>61.0</v>
       </c>
       <c r="D62" s="3" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="E62" s="19"/>
       <c r="F62" s="19"/>
@@ -10761,7 +10876,9 @@
       <c r="T62" s="19"/>
       <c r="U62" s="19"/>
       <c r="V62" s="19"/>
-      <c r="W62" s="19"/>
+      <c r="W62" s="7">
+        <v>0.923</v>
+      </c>
       <c r="X62" s="19"/>
     </row>
     <row r="63">
@@ -10775,7 +10892,7 @@
         <v>62.0</v>
       </c>
       <c r="D63" s="8" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="E63" s="21"/>
       <c r="F63" s="21"/>
@@ -10803,7 +10920,9 @@
       <c r="T63" s="21"/>
       <c r="U63" s="21"/>
       <c r="V63" s="21"/>
-      <c r="W63" s="21"/>
+      <c r="W63" s="12">
+        <v>0.923</v>
+      </c>
       <c r="X63" s="21"/>
     </row>
     <row r="64">
@@ -10817,7 +10936,7 @@
         <v>63.0</v>
       </c>
       <c r="D64" s="3" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="E64" s="19"/>
       <c r="F64" s="19"/>
@@ -10845,7 +10964,9 @@
       <c r="T64" s="19"/>
       <c r="U64" s="19"/>
       <c r="V64" s="19"/>
-      <c r="W64" s="19"/>
+      <c r="W64" s="7">
+        <v>0.833</v>
+      </c>
       <c r="X64" s="19"/>
     </row>
     <row r="65">

</xml_diff>